<commit_message>
Fix Object Repo key mismatches in TC Excel files and Object Repo
- 99 TC files updated with correct object names (120 replacements):
  BAI/BAM/CRAI/CRAM/DICOM → lowercase; Paired-End → Pairedend;
  Hybrid Selection → HybridSelection; Targeted-Capture → TargetedCapture;
  Illumina → ILLUMINA-Chkbx; Normal/Tumor-Chkbx → Normal/Tumor_Chkbx;
  Adenoma NOS / Colorectal Carcinoma → no-space versions;
  StudyDataTypes/Genomic_Chkbx → Genomic-Chkbx
- Added phs003163_Chkbx to CDS_ObjectRepository.xlsx

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ObjectRepository/CDS_ObjectRepository.xlsx
+++ b/ObjectRepository/CDS_ObjectRepository.xlsx
@@ -1550,7 +1550,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C385"/>
+  <dimension ref="A1:C386"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="55" customWidth="1" min="1" max="1"/>
@@ -8100,6 +8100,23 @@
       <c r="C385" s="2" t="inlineStr">
         <is>
           <t>(//*[@id="[object Object]"])[2]</t>
+        </is>
+      </c>
+    </row>
+    <row r="386">
+      <c r="A386" t="inlineStr">
+        <is>
+          <t>CDS/Data_page/Filter/StudyFacet/PHS_Accession/phs003163_Chkbx</t>
+        </is>
+      </c>
+      <c r="B386" t="inlineStr">
+        <is>
+          <t>phs003163_Chkbx</t>
+        </is>
+      </c>
+      <c r="C386" t="inlineStr">
+        <is>
+          <t>//*[@id="checkbox_PHS Accession_phs003163"]</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix missing Object Repo keys and TC Excel key mismatches
- Add LymphomaNOS_Chkbx and PrimaryXenograftTissue_Chkbx to CDS_ObjectRepository.xlsx
- Fix 31 TC Excel files: correct key names for InstrumentModel (IlluminaNovaSeq6000,
  IlluminaNovaSeqXPlus), ReferenceGenomeAssembly (Notspecifiedindata), SampleType
  (BloodDerivedNormal, Blood, DNA, RNA, Tissue, PrimaryXenograftTissue), and
  PrimaryDiagnosis (LymphomaNOS) across affected test cases

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ObjectRepository/CDS_ObjectRepository.xlsx
+++ b/ObjectRepository/CDS_ObjectRepository.xlsx
@@ -1550,7 +1550,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C386"/>
+  <dimension ref="A1:C388"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="55" customWidth="1" min="1" max="1"/>
@@ -8117,6 +8117,40 @@
       <c r="C386" t="inlineStr">
         <is>
           <t>//*[@id="checkbox_PHS Accession_phs003163"]</t>
+        </is>
+      </c>
+    </row>
+    <row r="387">
+      <c r="A387" t="inlineStr">
+        <is>
+          <t>CDS/Data_page/Filter/DiagnosisFacet/PrimaryDiagnosis/LymphomaNOS_Chkbx</t>
+        </is>
+      </c>
+      <c r="B387" t="inlineStr">
+        <is>
+          <t>LymphomaNOS_Chkbx</t>
+        </is>
+      </c>
+      <c r="C387" t="inlineStr">
+        <is>
+          <t>//*[@id="checkbox_PRIMARY DIAGNOSIS_Lymphoma, NOS"]</t>
+        </is>
+      </c>
+    </row>
+    <row r="388">
+      <c r="A388" t="inlineStr">
+        <is>
+          <t>CDS/Data_page/Filter/SamplesFacet/SampleType/PrimaryXenograftTissue_Chkbx</t>
+        </is>
+      </c>
+      <c r="B388" t="inlineStr">
+        <is>
+          <t>PrimaryXenograftTissue_Chkbx</t>
+        </is>
+      </c>
+      <c r="C388" t="inlineStr">
+        <is>
+          <t>//*[@id="checkbox_sample type_Primary Xenograft Tissue"]</t>
         </is>
       </c>
     </row>

</xml_diff>